<commit_message>
fixed images covering the cells' borders/outlines
</commit_message>
<xml_diff>
--- a/Imprimir.xlsx
+++ b/Imprimir.xlsx
@@ -1581,41 +1581,41 @@
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>BLD070</t>
+          <t>BLF037</t>
         </is>
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>10226359</t>
+          <t>10198819</t>
         </is>
       </c>
       <c r="C4" s="16" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>BOX</t>
+          <t>SLIVE</t>
         </is>
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
-          <t>0000118237</t>
+          <t>0000118236</t>
         </is>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>BLD074</t>
+          <t>BLE045</t>
         </is>
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>10226441</t>
+          <t>10208005</t>
         </is>
       </c>
       <c r="C5" s="16" t="n">
-        <v>10</v>
+        <v>180</v>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
@@ -1624,23 +1624,23 @@
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>0000118242</t>
+          <t>0000118255</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>BLD088</t>
+          <t>BLF079</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>10227896</t>
+          <t>10208005</t>
         </is>
       </c>
       <c r="C6" s="16" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
@@ -1649,123 +1649,123 @@
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>0000118243</t>
+          <t>0000118256</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>BLE003</t>
+          <t>BLH074</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>10226420</t>
+          <t>10208167</t>
         </is>
       </c>
       <c r="C7" s="16" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>SLIVE</t>
+          <t>SLEEVE P</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>0000118249</t>
+          <t>0000118258</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>BLE005</t>
+          <t>BLG003</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>10226386</t>
+          <t>10223108</t>
         </is>
       </c>
       <c r="C8" s="16" t="n">
-        <v>200</v>
+        <v>110</v>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>BOX</t>
+          <t>SLIVE</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>0000118267</t>
+          <t>0000118230</t>
         </is>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t>BLE006</t>
+          <t>BLH077</t>
         </is>
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>10226385</t>
+          <t>10223435</t>
         </is>
       </c>
       <c r="C9" s="16" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>SLIVE</t>
+          <t>BOX</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>0000118231</t>
+          <t>0000118227</t>
         </is>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>BLE015</t>
+          <t>BLH065</t>
         </is>
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>10226452</t>
+          <t>10223657</t>
         </is>
       </c>
       <c r="C10" s="16" t="n">
-        <v>80</v>
+        <v>170</v>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>SLEEVE P</t>
+          <t>BOX</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>0000118247</t>
+          <t>0000118235</t>
         </is>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>BLE024</t>
+          <t>BLF083</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>10226380</t>
+          <t>10224293</t>
         </is>
       </c>
       <c r="C11" s="16" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
@@ -1774,48 +1774,48 @@
       </c>
       <c r="E11" s="16" t="inlineStr">
         <is>
-          <t>0000118253</t>
+          <t>0000118233</t>
         </is>
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>BLE031</t>
+          <t>BLF089</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>10226367</t>
+          <t>10224293</t>
         </is>
       </c>
       <c r="C12" s="16" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>NINE</t>
+          <t>BOX</t>
         </is>
       </c>
       <c r="E12" s="16" t="inlineStr">
         <is>
-          <t>0000118259</t>
+          <t>0000118234</t>
         </is>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>BLE045</t>
+          <t>BLD070</t>
         </is>
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>10208005</t>
+          <t>10226359</t>
         </is>
       </c>
       <c r="C13" s="16" t="n">
-        <v>180</v>
+        <v>10</v>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
@@ -1824,39 +1824,39 @@
       </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
-          <t>0000118255</t>
+          <t>0000118237</t>
         </is>
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>BLF001</t>
+          <t>BLF043</t>
         </is>
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>10226404</t>
+          <t>10226361</t>
         </is>
       </c>
       <c r="C14" s="16" t="n">
-        <v>160</v>
+        <v>40</v>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>BOX</t>
+          <t>SLIVE</t>
         </is>
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
-          <t>0000118264</t>
+          <t>0000118232</t>
         </is>
       </c>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>BLF026</t>
+          <t>BLE031</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
@@ -1865,7 +1865,7 @@
         </is>
       </c>
       <c r="C15" s="16" t="n">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
@@ -1874,44 +1874,44 @@
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>0000118260</t>
+          <t>0000118259</t>
         </is>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>BLF037</t>
+          <t>BLF026</t>
         </is>
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>10198819</t>
+          <t>10226367</t>
         </is>
       </c>
       <c r="C16" s="16" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>SLIVE</t>
+          <t>NINE</t>
         </is>
       </c>
       <c r="E16" s="16" t="inlineStr">
         <is>
-          <t>0000118236</t>
+          <t>0000118260</t>
         </is>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>BLF043</t>
+          <t>FR.01.02.01.04</t>
         </is>
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>10226361</t>
+          <t>10226380</t>
         </is>
       </c>
       <c r="C17" s="16" t="n">
@@ -1919,28 +1919,28 @@
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>SLIVE</t>
+          <t>BOX</t>
         </is>
       </c>
       <c r="E17" s="16" t="inlineStr">
         <is>
-          <t>0000118232</t>
+          <t>0000118134</t>
         </is>
       </c>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>BLF051</t>
+          <t>BLH054</t>
         </is>
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>10226388</t>
+          <t>10226380</t>
         </is>
       </c>
       <c r="C18" s="16" t="n">
-        <v>30</v>
+        <v>340</v>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
@@ -1949,73 +1949,73 @@
       </c>
       <c r="E18" s="16" t="inlineStr">
         <is>
-          <t>0000118261</t>
+          <t>0000118252</t>
         </is>
       </c>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>BLF076</t>
+          <t>BLE024</t>
         </is>
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>10226403</t>
+          <t>10226380</t>
         </is>
       </c>
       <c r="C19" s="16" t="n">
-        <v>80</v>
+        <v>220</v>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>SLIVE</t>
+          <t>BOX</t>
         </is>
       </c>
       <c r="E19" s="16" t="inlineStr">
         <is>
-          <t>0000118245</t>
+          <t>0000118253</t>
         </is>
       </c>
     </row>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>BLF079</t>
+          <t>BLE006</t>
         </is>
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>10208005</t>
+          <t>10226385</t>
         </is>
       </c>
       <c r="C20" s="16" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D20" s="16" t="inlineStr">
         <is>
-          <t>BOX</t>
+          <t>SLIVE</t>
         </is>
       </c>
       <c r="E20" s="16" t="inlineStr">
         <is>
-          <t>0000118256</t>
+          <t>0000118231</t>
         </is>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>BLF083</t>
+          <t>FR.01.02.01.03</t>
         </is>
       </c>
       <c r="B21" s="16" t="inlineStr">
         <is>
-          <t>10224293</t>
+          <t>10226386</t>
         </is>
       </c>
       <c r="C21" s="16" t="n">
-        <v>120</v>
+        <v>20</v>
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
@@ -2024,23 +2024,23 @@
       </c>
       <c r="E21" s="16" t="inlineStr">
         <is>
-          <t>0000118233</t>
+          <t>0000118130</t>
         </is>
       </c>
     </row>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>BLF089</t>
+          <t>BLE005</t>
         </is>
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>10224293</t>
+          <t>10226386</t>
         </is>
       </c>
       <c r="C22" s="16" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
@@ -2049,73 +2049,73 @@
       </c>
       <c r="E22" s="16" t="inlineStr">
         <is>
-          <t>0000118234</t>
+          <t>0000118267</t>
         </is>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>BLG003</t>
+          <t>BLF051</t>
         </is>
       </c>
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>10223108</t>
+          <t>10226388</t>
         </is>
       </c>
       <c r="C23" s="16" t="n">
-        <v>110</v>
+        <v>30</v>
       </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
-          <t>SLIVE</t>
+          <t>BOX</t>
         </is>
       </c>
       <c r="E23" s="16" t="inlineStr">
         <is>
-          <t>0000118230</t>
+          <t>0000118261</t>
         </is>
       </c>
     </row>
     <row r="24" ht="45" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>BLG085</t>
+          <t>BLF076</t>
         </is>
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>10226454</t>
+          <t>10226403</t>
         </is>
       </c>
       <c r="C24" s="16" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="D24" s="16" t="inlineStr">
         <is>
-          <t>BOX</t>
+          <t>SLIVE</t>
         </is>
       </c>
       <c r="E24" s="16" t="inlineStr">
         <is>
-          <t>0000118241</t>
+          <t>0000118245</t>
         </is>
       </c>
     </row>
     <row r="25" ht="45" customHeight="1">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>BLH054</t>
+          <t>BLF001</t>
         </is>
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>10226380</t>
+          <t>10226404</t>
         </is>
       </c>
       <c r="C25" s="16" t="n">
-        <v>340</v>
+        <v>160</v>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
@@ -2124,82 +2124,82 @@
       </c>
       <c r="E25" s="16" t="inlineStr">
         <is>
-          <t>0000118252</t>
+          <t>0000118264</t>
         </is>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
-          <t>BLH065</t>
+          <t>BLE003</t>
         </is>
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>10223657</t>
+          <t>10226420</t>
         </is>
       </c>
       <c r="C26" s="16" t="n">
-        <v>170</v>
+        <v>10</v>
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>BOX</t>
+          <t>SLIVE</t>
         </is>
       </c>
       <c r="E26" s="16" t="inlineStr">
         <is>
-          <t>0000118235</t>
+          <t>0000118249</t>
         </is>
       </c>
     </row>
     <row r="27" ht="45" customHeight="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>BLH074</t>
+          <t>BLD074</t>
         </is>
       </c>
       <c r="B27" s="16" t="inlineStr">
         <is>
-          <t>10208167</t>
+          <t>10226441</t>
         </is>
       </c>
       <c r="C27" s="16" t="n">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>SLEEVE P</t>
+          <t>BOX</t>
         </is>
       </c>
       <c r="E27" s="16" t="inlineStr">
         <is>
-          <t>0000118258</t>
+          <t>0000118242</t>
         </is>
       </c>
     </row>
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>BLH077</t>
+          <t>BLE015</t>
         </is>
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
-          <t>10223435</t>
+          <t>10226452</t>
         </is>
       </c>
       <c r="C28" s="16" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="D28" s="16" t="inlineStr">
         <is>
-          <t>BOX</t>
+          <t>SLEEVE P</t>
         </is>
       </c>
       <c r="E28" s="16" t="inlineStr">
         <is>
-          <t>0000118227</t>
+          <t>0000118247</t>
         </is>
       </c>
     </row>
@@ -2231,16 +2231,16 @@
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="16" t="inlineStr">
         <is>
-          <t>FR.01.02.01.03</t>
+          <t>BLG085</t>
         </is>
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>10226386</t>
+          <t>10226454</t>
         </is>
       </c>
       <c r="C30" s="16" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
@@ -2249,23 +2249,23 @@
       </c>
       <c r="E30" s="16" t="inlineStr">
         <is>
-          <t>0000118130</t>
+          <t>0000118241</t>
         </is>
       </c>
     </row>
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="16" t="inlineStr">
         <is>
-          <t>FR.01.02.01.04</t>
+          <t>BLD088</t>
         </is>
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>10226380</t>
+          <t>10227896</t>
         </is>
       </c>
       <c r="C31" s="16" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="E31" s="16" t="inlineStr">
         <is>
-          <t>0000118134</t>
+          <t>0000118243</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
increased barcode size and switched rendering method
</commit_message>
<xml_diff>
--- a/Imprimir.xlsx
+++ b/Imprimir.xlsx
@@ -78,7 +78,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -130,11 +130,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
@@ -185,6 +194,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -192,7 +207,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="22">
     <dxf>
       <border>
         <left style="thin">
@@ -210,6 +225,26 @@
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -483,7 +518,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1485900" cy="561975"/>
+    <ext cx="2162175" cy="752475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -508,7 +543,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1485900" cy="561975"/>
+    <ext cx="2162175" cy="752475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -533,7 +568,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1485900" cy="561975"/>
+    <ext cx="2162175" cy="752475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -558,7 +593,7 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1485900" cy="561975"/>
+    <ext cx="2162175" cy="752475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -583,7 +618,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1485900" cy="561975"/>
+    <ext cx="2162175" cy="752475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -608,7 +643,7 @@
       <row>8</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1485900" cy="561975"/>
+    <ext cx="2162175" cy="752475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -633,7 +668,7 @@
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1485900" cy="561975"/>
+    <ext cx="2162175" cy="752475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
@@ -658,7 +693,7 @@
       <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1485900" cy="561975"/>
+    <ext cx="2162175" cy="752475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="8" name="Image 8" descr="Picture"/>
@@ -683,7 +718,7 @@
       <row>11</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1485900" cy="561975"/>
+    <ext cx="2162175" cy="752475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -708,7 +743,7 @@
       <row>12</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1485900" cy="561975"/>
+    <ext cx="2162175" cy="752475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -733,7 +768,7 @@
       <row>13</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1485900" cy="561975"/>
+    <ext cx="2162175" cy="752475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -741,431 +776,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>14</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="12" name="Image 12" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>15</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="13" name="Image 13" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>16</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="14" name="Image 14" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="15" name="Image 15" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>18</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>19</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>21</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>22</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="20" name="Image 20" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId20"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>23</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="21" name="Image 21" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId21"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>24</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="22" name="Image 22" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId22"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>25</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="23" name="Image 23" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId23"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>26</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="24" name="Image 24" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId24"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>27</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="25" name="Image 25" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId25"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>28</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="26" name="Image 26" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId26"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>29</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="27" name="Image 27" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId27"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>30</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1485900" cy="561975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="28" name="Image 28" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId28"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1508,7 +1118,7 @@
     <col width="9.140625" customWidth="1" style="16" min="3" max="3"/>
     <col width="9.5703125" bestFit="1" customWidth="1" style="16" min="4" max="4"/>
     <col width="11" bestFit="1" customWidth="1" style="16" min="5" max="5"/>
-    <col width="22" bestFit="1" customWidth="1" style="16" min="6" max="6"/>
+    <col width="32" bestFit="1" customWidth="1" style="16" min="6" max="6"/>
     <col width="9.140625" customWidth="1" style="16" min="7" max="16384"/>
   </cols>
   <sheetData>
@@ -1520,7 +1130,7 @@
       </c>
       <c r="B1" s="15" t="inlineStr">
         <is>
-          <t>6878107316</t>
+          <t>6878309021</t>
         </is>
       </c>
       <c r="C1" s="14" t="inlineStr">
@@ -1578,705 +1188,399 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="45" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>BLF037</t>
+          <t>BLF026</t>
         </is>
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>10198819</t>
+          <t>10226367</t>
         </is>
       </c>
       <c r="C4" s="16" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
+          <t>NINE</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>0000125501</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>BLF079</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>10226368</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>NINE</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>0000125500</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>BLG025</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>10226374</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>270</v>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>NINE</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
+        <is>
+          <t>0000125495</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>BLD074</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>10226374</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>NINE</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>0000125496</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>BLD069</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>10226398</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>240</v>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
           <t>SLIVE</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
-        <is>
-          <t>0000118236</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>BLE045</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>10208005</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="n">
-        <v>180</v>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>0000125502</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>BLD086</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>10226398</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>SLIVE</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>0000125503</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>BLE029</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>10226398</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>SLIVE</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>0000125504</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>FR.01.01.01.02</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>10226421</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>BOX</t>
         </is>
       </c>
-      <c r="E5" s="16" t="inlineStr">
-        <is>
-          <t>0000118255</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>BLF079</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>10208005</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="n">
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>0000125351</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>BLE013</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>10226422</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D12" s="16" t="inlineStr">
         <is>
           <t>BOX</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
-        <is>
-          <t>0000118256</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>BLH074</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>10208167</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="n">
-        <v>80</v>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>SLEEVE P</t>
-        </is>
-      </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>0000118258</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>BLG003</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>10223108</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="n">
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>0000125493</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>BLD081</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>10226422</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="n">
         <v>110</v>
       </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>SLIVE</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>0000118230</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>BLH077</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>10223435</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="n">
-        <v>30</v>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>BOX</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
-        <is>
-          <t>0000118227</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>BLH065</t>
-        </is>
-      </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>10223657</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="n">
-        <v>170</v>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E10" s="16" t="inlineStr">
-        <is>
-          <t>0000118235</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
-        <is>
-          <t>BLF083</t>
-        </is>
-      </c>
-      <c r="B11" s="16" t="inlineStr">
-        <is>
-          <t>10224293</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="n">
-        <v>120</v>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr">
-        <is>
-          <t>0000118233</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>BLF089</t>
-        </is>
-      </c>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>10224293</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="n">
-        <v>50</v>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E12" s="16" t="inlineStr">
-        <is>
-          <t>0000118234</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>BLD070</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>10226359</t>
-        </is>
-      </c>
-      <c r="C13" s="16" t="n">
-        <v>10</v>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
-          <t>0000118237</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="45" customHeight="1">
+          <t>0000125494</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>BLF043</t>
+          <t>BLF053</t>
         </is>
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>10226361</t>
+          <t>10247603</t>
         </is>
       </c>
       <c r="C14" s="16" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>SLIVE</t>
+          <t>NINE</t>
         </is>
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
-          <t>0000118232</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>BLE031</t>
-        </is>
-      </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>10226367</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="n">
-        <v>10</v>
-      </c>
-      <c r="D15" s="16" t="inlineStr">
-        <is>
-          <t>NINE</t>
-        </is>
-      </c>
-      <c r="E15" s="16" t="inlineStr">
-        <is>
-          <t>0000118259</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>BLF026</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>10226367</t>
-        </is>
-      </c>
-      <c r="C16" s="16" t="n">
-        <v>70</v>
-      </c>
-      <c r="D16" s="16" t="inlineStr">
-        <is>
-          <t>NINE</t>
-        </is>
-      </c>
-      <c r="E16" s="16" t="inlineStr">
-        <is>
-          <t>0000118260</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>FR.01.02.01.04</t>
-        </is>
-      </c>
-      <c r="B17" s="16" t="inlineStr">
-        <is>
-          <t>10226380</t>
-        </is>
-      </c>
-      <c r="C17" s="16" t="n">
-        <v>40</v>
-      </c>
-      <c r="D17" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E17" s="16" t="inlineStr">
-        <is>
-          <t>0000118134</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>BLH054</t>
-        </is>
-      </c>
-      <c r="B18" s="16" t="inlineStr">
-        <is>
-          <t>10226380</t>
-        </is>
-      </c>
-      <c r="C18" s="16" t="n">
-        <v>340</v>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E18" s="16" t="inlineStr">
-        <is>
-          <t>0000118252</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>BLE024</t>
-        </is>
-      </c>
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>10226380</t>
-        </is>
-      </c>
-      <c r="C19" s="16" t="n">
-        <v>220</v>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E19" s="16" t="inlineStr">
-        <is>
-          <t>0000118253</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>BLE006</t>
-        </is>
-      </c>
-      <c r="B20" s="16" t="inlineStr">
-        <is>
-          <t>10226385</t>
-        </is>
-      </c>
-      <c r="C20" s="16" t="n">
-        <v>10</v>
-      </c>
-      <c r="D20" s="16" t="inlineStr">
-        <is>
-          <t>SLIVE</t>
-        </is>
-      </c>
-      <c r="E20" s="16" t="inlineStr">
-        <is>
-          <t>0000118231</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>FR.01.02.01.03</t>
-        </is>
-      </c>
-      <c r="B21" s="16" t="inlineStr">
-        <is>
-          <t>10226386</t>
-        </is>
-      </c>
-      <c r="C21" s="16" t="n">
-        <v>20</v>
-      </c>
-      <c r="D21" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E21" s="16" t="inlineStr">
-        <is>
-          <t>0000118130</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="45" customHeight="1">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t>BLE005</t>
-        </is>
-      </c>
-      <c r="B22" s="16" t="inlineStr">
-        <is>
-          <t>10226386</t>
-        </is>
-      </c>
-      <c r="C22" s="16" t="n">
-        <v>200</v>
-      </c>
-      <c r="D22" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E22" s="16" t="inlineStr">
-        <is>
-          <t>0000118267</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="45" customHeight="1">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>BLF051</t>
-        </is>
-      </c>
-      <c r="B23" s="16" t="inlineStr">
-        <is>
-          <t>10226388</t>
-        </is>
-      </c>
-      <c r="C23" s="16" t="n">
-        <v>30</v>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E23" s="16" t="inlineStr">
-        <is>
-          <t>0000118261</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="45" customHeight="1">
-      <c r="A24" s="16" t="inlineStr">
-        <is>
-          <t>BLF076</t>
-        </is>
-      </c>
-      <c r="B24" s="16" t="inlineStr">
-        <is>
-          <t>10226403</t>
-        </is>
-      </c>
-      <c r="C24" s="16" t="n">
-        <v>80</v>
-      </c>
-      <c r="D24" s="16" t="inlineStr">
-        <is>
-          <t>SLIVE</t>
-        </is>
-      </c>
-      <c r="E24" s="16" t="inlineStr">
-        <is>
-          <t>0000118245</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="45" customHeight="1">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t>BLF001</t>
-        </is>
-      </c>
-      <c r="B25" s="16" t="inlineStr">
-        <is>
-          <t>10226404</t>
-        </is>
-      </c>
-      <c r="C25" s="16" t="n">
-        <v>160</v>
-      </c>
-      <c r="D25" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E25" s="16" t="inlineStr">
-        <is>
-          <t>0000118264</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="45" customHeight="1">
-      <c r="A26" s="16" t="inlineStr">
-        <is>
-          <t>BLE003</t>
-        </is>
-      </c>
-      <c r="B26" s="16" t="inlineStr">
-        <is>
-          <t>10226420</t>
-        </is>
-      </c>
-      <c r="C26" s="16" t="n">
-        <v>10</v>
-      </c>
-      <c r="D26" s="16" t="inlineStr">
-        <is>
-          <t>SLIVE</t>
-        </is>
-      </c>
-      <c r="E26" s="16" t="inlineStr">
-        <is>
-          <t>0000118249</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="45" customHeight="1">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t>BLD074</t>
-        </is>
-      </c>
-      <c r="B27" s="16" t="inlineStr">
-        <is>
-          <t>10226441</t>
-        </is>
-      </c>
-      <c r="C27" s="16" t="n">
-        <v>10</v>
-      </c>
-      <c r="D27" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E27" s="16" t="inlineStr">
-        <is>
-          <t>0000118242</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="45" customHeight="1">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>BLE015</t>
-        </is>
-      </c>
-      <c r="B28" s="16" t="inlineStr">
-        <is>
-          <t>10226452</t>
-        </is>
-      </c>
-      <c r="C28" s="16" t="n">
-        <v>80</v>
-      </c>
-      <c r="D28" s="16" t="inlineStr">
-        <is>
-          <t>SLEEVE P</t>
-        </is>
-      </c>
-      <c r="E28" s="16" t="inlineStr">
-        <is>
-          <t>0000118247</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="45" customHeight="1">
-      <c r="A29" s="16" t="inlineStr">
-        <is>
-          <t>BLH087</t>
-        </is>
-      </c>
-      <c r="B29" s="16" t="inlineStr">
-        <is>
-          <t>10226452</t>
-        </is>
-      </c>
-      <c r="C29" s="16" t="n">
-        <v>110</v>
-      </c>
-      <c r="D29" s="16" t="inlineStr">
-        <is>
-          <t>SLEEVE P</t>
-        </is>
-      </c>
-      <c r="E29" s="16" t="inlineStr">
-        <is>
-          <t>0000118248</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="45" customHeight="1">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>BLG085</t>
-        </is>
-      </c>
-      <c r="B30" s="16" t="inlineStr">
-        <is>
-          <t>10226454</t>
-        </is>
-      </c>
-      <c r="C30" s="16" t="n">
-        <v>40</v>
-      </c>
-      <c r="D30" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E30" s="16" t="inlineStr">
-        <is>
-          <t>0000118241</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="45" customHeight="1">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>BLD088</t>
-        </is>
-      </c>
-      <c r="B31" s="16" t="inlineStr">
-        <is>
-          <t>10227896</t>
-        </is>
-      </c>
-      <c r="C31" s="16" t="n">
-        <v>10</v>
-      </c>
-      <c r="D31" s="16" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E31" s="16" t="inlineStr">
-        <is>
-          <t>0000118243</t>
-        </is>
-      </c>
+          <t>0000125497</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="n"/>
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="16" t="n"/>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="16" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="n"/>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="16" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="n"/>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="16" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="n"/>
+      <c r="B18" s="16" t="n"/>
+      <c r="C18" s="16" t="n"/>
+      <c r="D18" s="16" t="n"/>
+      <c r="E18" s="16" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="n"/>
+      <c r="B19" s="16" t="n"/>
+      <c r="C19" s="16" t="n"/>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="16" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="n"/>
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="16" t="n"/>
+      <c r="D20" s="16" t="n"/>
+      <c r="E20" s="16" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="n"/>
+      <c r="B21" s="16" t="n"/>
+      <c r="C21" s="16" t="n"/>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="16" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="n"/>
+      <c r="B22" s="16" t="n"/>
+      <c r="C22" s="16" t="n"/>
+      <c r="D22" s="16" t="n"/>
+      <c r="E22" s="16" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="n"/>
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="16" t="n"/>
+      <c r="D23" s="16" t="n"/>
+      <c r="E23" s="16" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="n"/>
+      <c r="B24" s="16" t="n"/>
+      <c r="C24" s="16" t="n"/>
+      <c r="D24" s="16" t="n"/>
+      <c r="E24" s="16" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="n"/>
+      <c r="B25" s="16" t="n"/>
+      <c r="C25" s="16" t="n"/>
+      <c r="D25" s="16" t="n"/>
+      <c r="E25" s="16" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="n"/>
+      <c r="B26" s="16" t="n"/>
+      <c r="C26" s="16" t="n"/>
+      <c r="D26" s="16" t="n"/>
+      <c r="E26" s="16" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="n"/>
+      <c r="B27" s="16" t="n"/>
+      <c r="C27" s="16" t="n"/>
+      <c r="D27" s="16" t="n"/>
+      <c r="E27" s="16" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="n"/>
+      <c r="B28" s="16" t="n"/>
+      <c r="C28" s="16" t="n"/>
+      <c r="D28" s="16" t="n"/>
+      <c r="E28" s="16" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="n"/>
+      <c r="B29" s="16" t="n"/>
+      <c r="C29" s="16" t="n"/>
+      <c r="D29" s="16" t="n"/>
+      <c r="E29" s="16" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="n"/>
+      <c r="B30" s="16" t="n"/>
+      <c r="C30" s="16" t="n"/>
+      <c r="D30" s="16" t="n"/>
+      <c r="E30" s="16" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="n"/>
+      <c r="B31" s="16" t="n"/>
+      <c r="C31" s="16" t="n"/>
+      <c r="D31" s="16" t="n"/>
+      <c r="E31" s="16" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="16" t="n"/>

</xml_diff>